<commit_message>
Fiche RP-01 ZETES enrichie, ZETES en premier, bouton PowerPoint
</commit_message>
<xml_diff>
--- a/tableau-synthese-E5.xlsx
+++ b/tableau-synthese-E5.xlsx
@@ -37,7 +37,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B12" authorId="0">
+    <comment ref="B13" authorId="0">
       <text>
         <r>
           <rPr>
@@ -73,7 +73,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E13" authorId="0">
+    <comment ref="E12" authorId="0">
       <text>
         <r>
           <rPr>
@@ -173,6 +173,24 @@
     <t xml:space="preserve">RP-01</t>
   </si>
   <si>
+    <t xml:space="preserve">Déploiement de terminaux mobiles par MDM (SOTI)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZETES France, Antony</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Milieu professionnel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sept. 2023 - août 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RP-02</t>
+  </si>
+  <si>
     <t xml:space="preserve">Infrastructure Active Directory (Windows Server, DNS, DHCP, GPO)</t>
   </si>
   <si>
@@ -183,24 +201,6 @@
   </si>
   <si>
     <t xml:space="preserve">2025-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RP-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Déploiement de terminaux mobiles par MDM (SOTI)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZETES France, Antony</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Milieu professionnel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sept. 2023 - août 2025</t>
   </si>
   <si>
     <t xml:space="preserve">RP-03</t>
@@ -465,7 +465,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -477,7 +477,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -905,12 +905,14 @@
       <c r="E12" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
+      <c r="F12" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="H12" s="10"/>
-      <c r="I12" s="11" t="s">
-        <v>29</v>
-      </c>
+      <c r="I12" s="10"/>
       <c r="J12" s="11" t="s">
         <v>29</v>
       </c>
@@ -932,14 +934,12 @@
       <c r="E13" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="F13" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>29</v>
-      </c>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
       <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
+      <c r="I13" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="J13" s="11" t="s">
         <v>29</v>
       </c>
@@ -949,17 +949,17 @@
       <c r="A14" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="12" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
@@ -976,14 +976,14 @@
       <c r="A15" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="9" t="s">
         <v>38</v>
       </c>
       <c r="C15" s="10" t="s">
         <v>39</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>40</v>
@@ -1003,17 +1003,17 @@
       <c r="A16" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F16" s="11" t="s">
         <v>29</v>
@@ -1030,14 +1030,14 @@
       <c r="A17" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="9" t="s">
         <v>44</v>
       </c>
       <c r="C17" s="10" t="s">
         <v>45</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>46</v>

</xml_diff>